<commit_message>
feat(F-NAR-019): ATOM-DIF.ENE.001-02 Le ballon sous le drap
</commit_message>
<xml_diff>
--- a/stories/arbres/ATOM-DIF.ENE.001-02.xlsx
+++ b/stories/arbres/ATOM-DIF.ENE.001-02.xlsx
@@ -671,7 +671,7 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>jardin le jour du linge</t>
+          <t>jardin le jour du linge, clap clap, savon, abeille, pierre chaude, cerceau, ballon</t>
         </is>
       </c>
     </row>
@@ -841,7 +841,7 @@
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>Victorina veut faire rebondir le ballon sur la pierre chaude. Nino a de l'énergie. Le ballon se cache sous le drap. Ils jouent, ils attendent, Victorina demande à maman. Le ballon rebondit.</t>
+          <t>Le savon reste dans l'air. Le linge fait clap clap. Sur le bois, un éclat de piquet luit. Victorina veut le cerceau, maintenant. Nino court trop. Le cerceau tombe. Sourire parti. Papa s'accroupit. Elle refuse de foncer. Merci vécu. Le ballon roule sous le drap. Elle s'arrête. Un éclat de piquet tient sur le bois.</t>
         </is>
       </c>
     </row>
@@ -1184,17 +1184,17 @@
       </c>
       <c r="E2" s="2" t="inlineStr">
         <is>
-          <t>Une pince à linge tombe dans l'herbe. Toc. Elle est rouge. Elle est chaude. Le drap blanc cache le soleil. Puis il le rend. Ça sent le savon. Papa arrose un pot. Tu entends l'eau, Victorina ? Oui, papa. Maman chante tout bas. Le linge est presque sec. Une pierre attend dans l'herbe. Elle est ronde. Elle est chaude. En ce moment, Victorina s'assoit dessus. La pierre est douce. Elle tiédit le pantalon. Je veux le ballon. Sur la pierre. Il est près du bac. Une abeille visite une chaussette bleue. Elle part. Victorina prend le ballon. Il est un peu poudreux. Nino arrive dans le jardin. Il court un peu. Il saute. Il a de l'énergie. Beaucoup d'énergie. Il saute, maman. C'est son énergie. Ce n'est pas une faute. Nino court vers le ballon. Le ballon roule. Il se cache sous le drap blanc. Le ballon. Il est dessous. On le cherche ensemble ? Le drap bouge un peu. Nino saute encore. Victorina regarde maman.</t>
+          <t>Ça sent le savon, dehors. Le linge fait clap clap. Ça sent bon, papa. Tu le sens, le savon ? Oui, papa. Un drap blanc tape un peu. Le drap est presque sec. Il tape, maman. Papa arrose un pot. De l'eau brille sur la terre. Tu entends l'eau, Victorina ? Oui, l'eau. Maman pose une pince rouge. Elle fait toc, près du fil. Un piquet tient le fil. Le bois est chaud, un peu rêche. Sur le bois, un éclat de piquet luit. Il brille, maman. Tu le vois, sur le piquet ? Oui, un petit point. Le soleil le touche. Une pierre ronde attend dans l'herbe. Elle tiédit le pantalon. Elle est chaude. Tu t'assois, Victorina ? Un peu. Une abeille visite une chaussette bleue. Elle fait un petit bzz. Elle part. L'abeille a fini. Le cerceau jaune dort près du bac. En ce moment, Victorina le prend. Je veux le cerceau, maintenant ! Tout de suite ? Oui, papa. Le plastique est tiède, un peu poudreux. Tu le fais rouler ? Oui, maman. Nino arrive dans le jardin. Il court trop. Il saute près du drap. Le cerceau ! Tu viens, Nino ? Oui. Victorina pousse le cerceau trop vite. Nino court dessus. Le cerceau tombe dans l'herbe. Il ne tourne plus. Oh. Il est tombé. Le sourire de Victorina disparaît. Dans sa poitrine, ça se bouscule. L'envie et la peur se heurtent. Ses épaules tombent un peu. Papa s'accroupit à la même hauteur. Tu vois Nino, Victorina ? Oui, papa. Tes mains sont chaudes, Victorina ? Un peu, maman. L'éclat de piquet tremble, puis tient.</t>
         </is>
       </c>
       <c r="F2" s="2" t="inlineStr">
         <is>
-          <t>Une pince à linge tombe dans l'herbe. Toc. Elle est rouge. Elle est chaude. Le drap blanc cache le soleil. Puis il le rend. Ça sent le savon. Papa arrose un pot. Tu entends l'eau, Victorina ? Oui, papa. Maman chante tout bas. Le linge est presque sec. Une pierre attend dans l'herbe. Elle est ronde. Elle est chaude. En ce moment, Victorina s'assoit dessus. La pierre est douce. Elle tiédit le pantalon. Je veux le ballon. Sur la pierre. Il est près du bac. Une abeille visite une chaussette bleue. Elle part. Victorina prend le ballon. Il est un peu poudreux. Nino arrive dans le jardin. Il court un peu. Il saute. Il a de l'énergie. Beaucoup d'énergie. Il saute, maman. C'est son énergie. Ce n'est pas une faute. Nino court vers le ballon. Le ballon roule. Il se cache sous le drap blanc. Le ballon. Il est dessous. On le cherche ensemble ? Le drap bouge un peu. Nino saute encore. Victorina regarde maman.</t>
+          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;Ça sent le savon, dehors. Le linge fait clap clap. Ça sent bon, papa. Tu le sens, le savon ? Oui, papa. Un drap blanc tape un peu. Le drap est presque sec. Il tape, maman. Papa arrose un pot. De l'eau brille sur la terre. Tu entends l'eau, Victorina ? Oui, l'eau. Maman pose une pince rouge. Elle fait toc, près du fil. Un piquet tient le fil. Le bois est chaud, un peu rêche. Sur le bois, un &lt;emphasis level="moderate"&gt;éclat de piquet&lt;/emphasis&gt; luit. Il brille, maman. Tu le vois, sur le piquet ? Oui, un petit point. Le soleil le touche. Une pierre ronde attend dans l'herbe. Elle tiédit le pantalon. Elle est chaude. Tu t'assois, Victorina ? Un peu. Une abeille visite une chaussette bleue. Elle fait un petit bzz. Elle part. L'abeille a fini. Le cerceau jaune dort près du bac. En ce moment, Victorina le prend. Je veux le cerceau, maintenant ! Tout de suite ? Oui, papa. Le plastique est tiède, un peu poudreux. Tu le fais rouler ? Oui, maman. Nino arrive dans le jardin. Il court trop. Il saute près du drap. Le cerceau ! Tu viens, Nino ? Oui. Victorina pousse le cerceau trop vite. Nino court dessus. Le cerceau tombe dans l'herbe. Il ne tourne plus. Oh. Il est tombé. Le sourire de Victorina disparaît. Dans sa poitrine, ça se bouscule. L'envie et la peur se heurtent. Ses épaules tombent un peu. Papa s'accroupit à la même hauteur. Tu vois Nino, Victorina ? Oui, papa. Tes mains sont chaudes, Victorina ? Un peu, maman. L'éclat de piquet tremble, puis tient.&lt;/prosody&gt;&lt;break time="560ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G2" s="2" t="inlineStr">
         <is>
-          <t>&lt;slow&gt;Sara est dans le jardin. Maman est là. Adam arrive. Adam court un peu. Il saute. Il a de l'&lt;emphasis&gt;énergie&lt;/emphasis&gt;. Beaucoup d'énergie. Ce n'est pas une faute. Sara le regarde. Maman dit : on peut jouer. On peut attendre. On peut demander à un adulte. Sara prend un cerceau. Elle dit : tu viens. Adam dit : oui. Ils jouent. Adam fait tourner le cerceau. Sara attend son tour. Adam pose le cerceau. Sara joue. Adam saute encore. L'énergie est là. Ce n'est pas une faute. Sara dit : on attend. Adam souffle. Il attend. Puis maman sort un ballon. Adam court vers le ballon. Sara va vers maman. Elle demande à un adulte. Maman dit : on se passe le ballon. Adam s'arrête. Il tend les mains. Sara envoie le ballon. Adam le renvoie. Ils jouent. Ils attendent, un peu. Maman dit : bravo. Adam a de l'énergie. Ce n'est pas une faute. On peut jouer. On peut attendre. Sara rit. Adam rit. Le cerceau reste dans l'herbe. Le ballon aussi. Maman dit encore : si c'est trop, on vient me voir. Sara hoche la tête. Adam hoche la tête. Ils se passent le ballon, tout près.&lt;/slow&gt; [pause]</t>
+          <t>Ça sent le savon, dehors. Le linge fait clap clap. Ça sent bon, papa. Tu le sens, le savon ? Oui, papa. Un drap blanc tape un peu. Le drap est presque sec. Il tape, maman. Papa arrose un pot. De l'eau brille sur la terre. Tu entends l'eau, Victorina ? Oui, l'eau. Maman pose une pince rouge. Elle fait toc, près du fil. Un piquet tient le fil. Le bois est chaud, un peu rêche. Sur le bois, un &lt;emphasis&gt;éclat de piquet&lt;/emphasis&gt; luit. Il brille, maman. Tu le vois, sur le piquet ? Oui, un petit point. Le soleil le touche. Une pierre ronde attend dans l'herbe. Elle tiédit le pantalon. Elle est chaude. Tu t'assois, Victorina ? Un peu. Une abeille visite une chaussette bleue. Elle fait un petit bzz. Elle part. L'abeille a fini. Le cerceau jaune dort près du bac. En ce moment, Victorina le prend. Je veux le cerceau, maintenant ! Tout de suite ? Oui, papa. Le plastique est tiède, un peu poudreux. Tu le fais rouler ? Oui, maman. Nino arrive dans le jardin. Il court trop. Il saute près du drap. Le cerceau ! Tu viens, Nino ? Oui. Victorina pousse le cerceau trop vite. Nino court dessus. Le cerceau tombe dans l'herbe. Il ne tourne plus. Oh. Il est tombé. Le sourire de Victorina disparaît. Dans sa poitrine, ça se bouscule. L'envie et la peur se heurtent. Ses épaules tombent un peu. Papa s'accroupit à la même hauteur. Tu vois Nino, Victorina ? Oui, papa. Tes mains sont chaudes, Victorina ? Un peu, maman. L'éclat de piquet tremble, puis tient. [pause]</t>
         </is>
       </c>
       <c r="H2" s="2" t="inlineStr"/>
@@ -1241,18 +1241,18 @@
         </is>
       </c>
       <c r="Y2" s="2" t="n">
-        <v>118</v>
+        <v>124</v>
       </c>
       <c r="Z2" s="2" t="inlineStr">
         <is>
-          <t>slow</t>
+          <t>medium</t>
         </is>
       </c>
       <c r="AA2" s="2" t="n">
-        <v>0.86</v>
+        <v>0.9</v>
       </c>
       <c r="AB2" s="2" t="n">
-        <v>1.28</v>
+        <v>1.22</v>
       </c>
       <c r="AC2" s="2" t="inlineStr">
         <is>
@@ -1275,30 +1275,30 @@
       </c>
       <c r="AH2" s="2" t="inlineStr">
         <is>
-          <t>énergie</t>
+          <t>éclat de piquet</t>
         </is>
       </c>
       <c r="AI2" s="2" t="n">
         <v>0</v>
       </c>
       <c r="AJ2" s="2" t="n">
-        <v>400</v>
+        <v>560</v>
       </c>
       <c r="AK2" s="2" t="n">
-        <v>380</v>
+        <v>300</v>
       </c>
       <c r="AL2" s="2" t="inlineStr">
         <is>
-          <t>calm</t>
+          <t>warm</t>
         </is>
       </c>
       <c r="AM2" s="2" t="inlineStr">
         <is>
-          <t>level</t>
+          <t>storytelling</t>
         </is>
       </c>
       <c r="AN2" s="2" t="n">
-        <v>0.333</v>
+        <v>0.34</v>
       </c>
       <c r="AO2" s="2" t="inlineStr"/>
       <c r="AP2" s="2" t="inlineStr">
@@ -1307,10 +1307,10 @@
         </is>
       </c>
       <c r="AQ2" s="2" t="n">
-        <v>0.86</v>
+        <v>0.9</v>
       </c>
       <c r="AR2" s="2" t="n">
-        <v>0.86</v>
+        <v>0.9</v>
       </c>
       <c r="AS2" s="2" t="n">
         <v>100</v>
@@ -1319,53 +1319,75 @@
         <v>50</v>
       </c>
       <c r="AU2" s="2" t="n">
-        <v>12</v>
-      </c>
-      <c r="AV2" s="2" t="inlineStr"/>
+        <v>8</v>
+      </c>
+      <c r="AV2" s="2" t="inlineStr">
+        <is>
+          <t>arc=installation; intention=émerveiller puis tendre; emotion=impatience puis découragement; intensite=2; destinataire=enfant; sous_texte=elle_veut_le_cerceau_maintenant; tempo=posé puis resserré; sourire=léger puis aucun; respiration=ample puis retenue</t>
+        </is>
+      </c>
       <c r="AW2" t="inlineStr">
         <is>
-          <t>narrateur|Une pince à linge tombe dans l'herbe.
-narrateur|Toc.
-narrateur|Elle est rouge.
-narrateur|Elle est chaude.
-narrateur|Le drap blanc cache le soleil.
-narrateur|Puis il le rend.
-narrateur|Ça sent le savon.
+          <t>narrateur|Ça sent le savon, dehors.
+narrateur|Le linge fait clap clap.
+enfant-f|Ça sent bon, papa.
+papa|Tu le sens, le savon ?
+enfant-f|Oui, papa.
+narrateur|Un drap blanc tape un peu.
+maman|Le drap est presque sec.
+enfant-f|Il tape, maman.
 narrateur|Papa arrose un pot.
+narrateur|De l'eau brille sur la terre.
 papa|Tu entends l'eau, Victorina ?
+enfant-f|Oui, l'eau.
+narrateur|Maman pose une pince rouge.
+narrateur|Elle fait toc, près du fil.
+narrateur|Un piquet tient le fil.
+narrateur|Le bois est chaud, un peu rêche.
+narrateur|Sur le bois, un éclat de piquet luit.
+enfant-f|Il brille, maman.
+maman|Tu le vois, sur le piquet ?
+enfant-f|Oui, un petit point.
+papa|Le soleil le touche.
+narrateur|Une pierre ronde attend dans l'herbe.
+narrateur|Elle tiédit le pantalon.
+enfant-f|Elle est chaude.
+maman|Tu t'assois, Victorina ?
+enfant-f|Un peu.
+narrateur|Une abeille visite une chaussette bleue.
+narrateur|Elle fait un petit bzz.
+enfant-f|Elle part.
+papa|L'abeille a fini.
+narrateur|Le cerceau jaune dort près du bac.
+narrateur|En ce moment, Victorina le prend.
+enfant-f|Je veux le cerceau, maintenant !
+papa|Tout de suite ?
 enfant-f|Oui, papa.
-narrateur|Maman chante tout bas.
-maman|Le linge est presque sec.
-narrateur|Une pierre attend dans l'herbe.
-narrateur|Elle est ronde.
-narrateur|Elle est chaude.
-narrateur|En ce moment, Victorina s'assoit dessus.
-narrateur|La pierre est douce.
-narrateur|Elle tiédit le pantalon.
-enfant-f|Je veux le ballon.
-enfant-f|Sur la pierre.
-maman|Il est près du bac.
-narrateur|Une abeille visite une chaussette bleue.
-narrateur|Elle part.
-narrateur|Victorina prend le ballon.
-narrateur|Il est un peu poudreux.
+narrateur|Le plastique est tiède, un peu poudreux.
+maman|Tu le fais rouler ?
+enfant-f|Oui, maman.
 narrateur|Nino arrive dans le jardin.
-narrateur|Il court un peu.
-narrateur|Il saute.
-narrateur|Il a de l'énergie.
-narrateur|Beaucoup d'énergie.
-enfant-f|Il saute, maman.
-maman|C'est son énergie.
-maman|Ce n'est pas une faute.
-narrateur|Nino court vers le ballon.
-narrateur|Le ballon roule.
-narrateur|Il se cache sous le drap blanc.
-enfant-f|Le ballon.
-enfant-f|Il est dessous.
-papa|On le cherche ensemble ?
-narrateur|Le drap bouge un peu.
-narrateur|Nino saute encore.
-narrateur|Victorina regarde maman.</t>
+narrateur|Il court trop.
+narrateur|Il saute près du drap.
+copain|Le cerceau !
+enfant-f|Tu viens, Nino ?
+copain|Oui.
+narrateur|Victorina pousse le cerceau trop vite.
+narrateur|Nino court dessus.
+narrateur|Le cerceau tombe dans l'herbe.
+narrateur|Il ne tourne plus.
+enfant-f|Oh.
+copain|Il est tombé.
+narrateur|Le sourire de Victorina disparaît.
+narrateur|Dans sa poitrine, ça se bouscule.
+narrateur|L'envie et la peur se heurtent.
+narrateur|Ses épaules tombent un peu.
+narrateur|Papa s'accroupit à la même hauteur.
+papa|Tu vois Nino, Victorina ?
+enfant-f|Oui, papa.
+maman|Tes mains sont chaudes, Victorina ?
+enfant-f|Un peu, maman.
+narrateur|L'éclat de piquet tremble, puis tient.</t>
         </is>
       </c>
       <c r="AX2" t="inlineStr">
@@ -1402,12 +1424,12 @@
       </c>
       <c r="F3" s="2" t="inlineStr">
         <is>
-          <t>Nino a de l'énergie. Que fait-on ?</t>
+          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="medium"&gt;Nino a de l'&lt;emphasis level="moderate"&gt;énergie&lt;/emphasis&gt;. Que fait-on ?&lt;/prosody&gt;&lt;break time="780ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G3" s="2" t="inlineStr">
         <is>
-          <t>&lt;slow&gt;Adam a de l'&lt;emphasis&gt;énergie&lt;/emphasis&gt;. Que fait-on ?&lt;/slow&gt;</t>
+          <t>&lt;soft&gt;&lt;slow&gt;Nino a de l'&lt;emphasis&gt;énergie&lt;/emphasis&gt;. Que fait-on ?&lt;/slow&gt;&lt;/soft&gt; [pause]</t>
         </is>
       </c>
       <c r="H3" s="2" t="inlineStr">
@@ -1470,7 +1492,7 @@
         </is>
       </c>
       <c r="Y3" s="2" t="n">
-        <v>100</v>
+        <v>104</v>
       </c>
       <c r="Z3" s="2" t="inlineStr">
         <is>
@@ -1481,7 +1503,7 @@
         <v>0.8</v>
       </c>
       <c r="AB3" s="2" t="n">
-        <v>1.4</v>
+        <v>1.36</v>
       </c>
       <c r="AC3" s="2" t="inlineStr">
         <is>
@@ -1496,11 +1518,11 @@
       <c r="AE3" s="2" t="inlineStr"/>
       <c r="AF3" s="2" t="inlineStr">
         <is>
-          <t>medium</t>
+          <t>soft</t>
         </is>
       </c>
       <c r="AG3" s="2" t="n">
-        <v>0</v>
+        <v>-2</v>
       </c>
       <c r="AH3" s="2" t="inlineStr">
         <is>
@@ -1511,23 +1533,23 @@
         <v>200</v>
       </c>
       <c r="AJ3" s="2" t="n">
-        <v>250</v>
+        <v>780</v>
       </c>
       <c r="AK3" s="2" t="n">
-        <v>380</v>
+        <v>360</v>
       </c>
       <c r="AL3" s="2" t="inlineStr">
         <is>
-          <t>warm</t>
+          <t>focused</t>
         </is>
       </c>
       <c r="AM3" s="2" t="inlineStr">
         <is>
-          <t>rise</t>
+          <t>rising</t>
         </is>
       </c>
       <c r="AN3" s="2" t="n">
-        <v>0.333</v>
+        <v>0.3</v>
       </c>
       <c r="AO3" s="2" t="inlineStr"/>
       <c r="AP3" s="2" t="inlineStr">
@@ -1542,7 +1564,7 @@
         <v>0.8</v>
       </c>
       <c r="AS3" s="2" t="n">
-        <v>100</v>
+        <v>82</v>
       </c>
       <c r="AT3" s="2" t="n">
         <v>50</v>
@@ -1552,7 +1574,7 @@
       </c>
       <c r="AV3" s="2" t="inlineStr">
         <is>
-          <t>question d'écoute, ne change pas le cours</t>
+          <t>arc=indice; intention=faire_deviner; emotion=attention; intensite=1; destinataire=enfant; sous_texte=nino_court_trop_que_fait_on; tempo=suspendu; sourire=aucun; respiration=courte_avant_question</t>
         </is>
       </c>
       <c r="AW3" t="inlineStr">
@@ -1585,17 +1607,17 @@
       </c>
       <c r="E4" s="2" t="inlineStr">
         <is>
-          <t>Victorina va vers maman. Maman, le ballon ? On joue avec le ballon. Ou on attend un peu. Tu viens me voir, si tu veux. On soulève le drap. Le drap sent le savon. Le ballon est là. Il est un peu tiède. Nino tend les mains. Il a encore de l'énergie. Ce n'est pas une faute. On attend. Nino souffle. Il attend. C'est à Victorina. Victorina pose le ballon sur la pierre. Poumf. Le ballon rebondit. Nino le rattrape. Il le rend. Ils jouent. Ils se passent le ballon. Tout près. L'herbe chatouille les genoux. Le ballon est bien gonflé ? Oui, papa. On reste encore un peu ? Encore un peu. Nino saute encore un peu. On peut attendre. Nino pose le ballon. Il attend son tour. Chacun son tour.</t>
+          <t>Victorina veut le cerceau, tout de suite. Je pousse, maintenant ! Elle avance trop vite vers Nino. Les mots se bousculent dans sa bouche. Attends. Nino recule d'un pas. Oh. Le sourire ne revient pas. Victorina refuse de foncer. Elle referme la bouche. Personne ne parle. Elle observe le cerceau, un instant. Elle écoute le clap clap du linge. Tu veux le cerceau avec Nino ? Papa reste à la même hauteur. Tu tiens le bord ? Nino ne dit rien, d'abord. Il pose les mains sur le plastique. Je le tiens. D'accord. Merci, Victorina. Papa a vu les deux, près du piquet. Le savon colle un peu, sous les doigts. Il est tiède. Ils essuient le cerceau sur l'herbe. Nino tient le bord, plus près. Le cerceau redevient plus léger, cette fois. Il tourne ! Oui. Tu le vois, le cerceau ? Oui, papa. Au milieu, Nino ? J'y vais. Victorina pousse, sans se presser. Nino suit le cerceau des yeux. Le cerceau danse une fois. Un. Deux. Le ventre de Victorina se desserre. Les épaules se relèvent un peu. On reste près du linge ? Oui. Tes mains sont au chaud ? Un peu, maman.</t>
         </is>
       </c>
       <c r="F4" s="2" t="inlineStr">
         <is>
-          <t>Victorina va vers maman. Maman, le ballon ? On joue avec le ballon. Ou on attend un peu. Tu viens me voir, si tu veux. On soulève le drap. Le drap sent le savon. Le ballon est là. Il est un peu tiède. Nino tend les mains. Il a encore de l'énergie. Ce n'est pas une faute. On attend. Nino souffle. Il attend. C'est à Victorina. Victorina pose le ballon sur la pierre. Poumf. Le ballon rebondit. Nino le rattrape. Il le rend. Ils jouent. Ils se passent le ballon. Tout près. L'herbe chatouille les genoux. Le ballon est bien gonflé ? Oui, papa. On reste encore un peu ? Encore un peu. Nino saute encore un peu. On peut attendre. Nino pose le ballon. Il attend son tour. Chacun son tour.</t>
+          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;Victorina veut le &lt;emphasis level="moderate"&gt;cerceau&lt;/emphasis&gt;, tout de suite. Je pousse, maintenant ! Elle avance trop vite vers Nino. Les mots se bousculent dans sa bouche. Attends. Nino recule d'un pas. Oh. Le sourire ne revient pas. Victorina refuse de foncer. Elle referme la bouche. Personne ne parle. Elle observe le cerceau, un instant. Elle écoute le clap clap du linge. Tu veux le cerceau avec Nino ? Papa reste à la même hauteur. Tu tiens le bord ? Nino ne dit rien, d'abord. Il pose les mains sur le plastique. Je le tiens. D'accord. Merci, Victorina. Papa a vu les deux, près du piquet. Le savon colle un peu, sous les doigts. Il est tiède. Ils essuient le cerceau sur l'herbe. Nino tient le bord, plus près. Le cerceau redevient plus léger, cette fois. Il tourne ! Oui. Tu le vois, le cerceau ? Oui, papa. Au milieu, Nino ? J'y vais. Victorina pousse, sans se presser. Nino suit le cerceau des yeux. Le cerceau danse une fois. Un. Deux. Le ventre de Victorina se desserre. Les épaules se relèvent un peu. On reste près du linge ? Oui. Tes mains sont au chaud ? Un peu, maman.&lt;/prosody&gt;&lt;break time="620ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G4" s="2" t="inlineStr">
         <is>
-          <t>&lt;slow&gt;Adam a de l'&lt;emphasis&gt;énergie&lt;/emphasis&gt;. Ce n'est pas une faute. Sara a joué. Elle a su attendre.&lt;/slow&gt; [pause]</t>
+          <t>Victorina veut le &lt;emphasis&gt;cerceau&lt;/emphasis&gt;, tout de suite. Je pousse, maintenant ! Elle avance trop vite vers Nino. Les mots se bousculent dans sa bouche. Attends. Nino recule d'un pas. Oh. Le sourire ne revient pas. Victorina refuse de foncer. Elle referme la bouche. Personne ne parle. Elle observe le cerceau, un instant. Elle écoute le clap clap du linge. Tu veux le cerceau avec Nino ? Papa reste à la même hauteur. Tu tiens le bord ? Nino ne dit rien, d'abord. Il pose les mains sur le plastique. Je le tiens. D'accord. Merci, Victorina. Papa a vu les deux, près du piquet. Le savon colle un peu, sous les doigts. Il est tiède. Ils essuient le cerceau sur l'herbe. Nino tient le bord, plus près. Le cerceau redevient plus léger, cette fois. Il tourne ! Oui. Tu le vois, le cerceau ? Oui, papa. Au milieu, Nino ? J'y vais. Victorina pousse, sans se presser. Nino suit le cerceau des yeux. Le cerceau danse une fois. Un. Deux. Le ventre de Victorina se desserre. Les épaules se relèvent un peu. On reste près du linge ? Oui. Tes mains sont au chaud ? Un peu, maman. [pause]</t>
         </is>
       </c>
       <c r="H4" s="2" t="inlineStr"/>
@@ -1642,18 +1664,18 @@
         </is>
       </c>
       <c r="Y4" s="2" t="n">
-        <v>118</v>
+        <v>122</v>
       </c>
       <c r="Z4" s="2" t="inlineStr">
         <is>
-          <t>slow</t>
+          <t>medium</t>
         </is>
       </c>
       <c r="AA4" s="2" t="n">
-        <v>0.86</v>
+        <v>0.88</v>
       </c>
       <c r="AB4" s="2" t="n">
-        <v>1.28</v>
+        <v>1.24</v>
       </c>
       <c r="AC4" s="2" t="inlineStr">
         <is>
@@ -1676,30 +1698,30 @@
       </c>
       <c r="AH4" s="2" t="inlineStr">
         <is>
-          <t>énergie</t>
+          <t>cerceau</t>
         </is>
       </c>
       <c r="AI4" s="2" t="n">
         <v>200</v>
       </c>
       <c r="AJ4" s="2" t="n">
-        <v>450</v>
+        <v>620</v>
       </c>
       <c r="AK4" s="2" t="n">
-        <v>380</v>
+        <v>310</v>
       </c>
       <c r="AL4" s="2" t="inlineStr">
         <is>
-          <t>calm</t>
+          <t>bright</t>
         </is>
       </c>
       <c r="AM4" s="2" t="inlineStr">
         <is>
-          <t>level</t>
+          <t>falling</t>
         </is>
       </c>
       <c r="AN4" s="2" t="n">
-        <v>0.333</v>
+        <v>0.33</v>
       </c>
       <c r="AO4" s="2" t="inlineStr"/>
       <c r="AP4" s="2" t="inlineStr">
@@ -1708,10 +1730,10 @@
         </is>
       </c>
       <c r="AQ4" s="2" t="n">
-        <v>0.86</v>
+        <v>0.88</v>
       </c>
       <c r="AR4" s="2" t="n">
-        <v>0.86</v>
+        <v>0.88</v>
       </c>
       <c r="AS4" s="2" t="n">
         <v>100</v>
@@ -1720,49 +1742,59 @@
         <v>50</v>
       </c>
       <c r="AU4" s="2" t="n">
-        <v>12</v>
+        <v>8</v>
       </c>
       <c r="AV4" s="2" t="inlineStr">
         <is>
-          <t>confirmation ; le moteur peut dire engine_ok/near avant ce chunk</t>
+          <t>arc=résolution; intention=faire_vivre_le_geste; emotion=retenue puis fierté_calme; intensite=2; destinataire=enfant; sous_texte=elle_refuse_de_foncer_ils_tiennent; tempo=posé; sourire=léger; respiration=relâchée</t>
         </is>
       </c>
       <c r="AW4" t="inlineStr">
         <is>
-          <t>narrateur|Victorina va vers maman.
-enfant-f|Maman, le ballon ?
-maman|On joue avec le ballon.
-maman|Ou on attend un peu.
-maman|Tu viens me voir, si tu veux.
-papa|On soulève le drap.
-narrateur|Le drap sent le savon.
-narrateur|Le ballon est là.
-narrateur|Il est un peu tiède.
-narrateur|Nino tend les mains.
-narrateur|Il a encore de l'énergie.
-maman|Ce n'est pas une faute.
-enfant-f|On attend.
-narrateur|Nino souffle.
-narrateur|Il attend.
-papa|C'est à Victorina.
-narrateur|Victorina pose le ballon sur la pierre.
-narrateur|Poumf.
-narrateur|Le ballon rebondit.
-narrateur|Nino le rattrape.
-narrateur|Il le rend.
-narrateur|Ils jouent.
-narrateur|Ils se passent le ballon.
-narrateur|Tout près.
-narrateur|L'herbe chatouille les genoux.
-papa|Le ballon est bien gonflé ?
+          <t>narrateur|Victorina veut le cerceau, tout de suite.
+enfant-f|Je pousse, maintenant !
+narrateur|Elle avance trop vite vers Nino.
+narrateur|Les mots se bousculent dans sa bouche.
+copain|Attends.
+narrateur|Nino recule d'un pas.
+enfant-f|Oh.
+narrateur|Le sourire ne revient pas.
+narrateur|Victorina refuse de foncer.
+narrateur|Elle referme la bouche.
+narrateur|Personne ne parle.
+narrateur|Elle observe le cerceau, un instant.
+narrateur|Elle écoute le clap clap du linge.
+papa|Tu veux le cerceau avec Nino ?
+narrateur|Papa reste à la même hauteur.
+enfant-f|Tu tiens le bord ?
+narrateur|Nino ne dit rien, d'abord.
+narrateur|Il pose les mains sur le plastique.
+copain|Je le tiens.
+enfant-f|D'accord.
+papa|Merci, Victorina.
+narrateur|Papa a vu les deux, près du piquet.
+maman|Le savon colle un peu, sous les doigts.
+enfant-f|Il est tiède.
+narrateur|Ils essuient le cerceau sur l'herbe.
+narrateur|Nino tient le bord, plus près.
+narrateur|Le cerceau redevient plus léger, cette fois.
+enfant-f|Il tourne !
+copain|Oui.
+papa|Tu le vois, le cerceau ?
 enfant-f|Oui, papa.
-maman|On reste encore un peu ?
-enfant-f|Encore un peu.
-narrateur|Nino saute encore un peu.
-enfant-f|On peut attendre.
-narrateur|Nino pose le ballon.
-narrateur|Il attend son tour.
-maman|Chacun son tour.</t>
+maman|Au milieu, Nino ?
+copain|J'y vais.
+narrateur|Victorina pousse, sans se presser.
+narrateur|Nino suit le cerceau des yeux.
+narrateur|Le cerceau danse une fois.
+copain|Un.
+enfant-f|Deux.
+narrateur|Le ventre de Victorina se desserre.
+narrateur|Les épaules se relèvent un peu.
+papa|On reste près du linge ?
+enfant-f|Oui.
+maman|Tes mains sont au chaud ?
+enfant-f|Un peu, maman.</t>
         </is>
       </c>
       <c r="AX4" t="inlineStr">
@@ -1794,17 +1826,17 @@
       </c>
       <c r="E5" s="2" t="inlineStr">
         <is>
-          <t>On rentre ? Oui, maman. Victorina porte le ballon. Nino ramasse la pince rouge. Vous vous dites merci ? Merci, Nino. Merci. Le linge fait encore clap clap. Le ballon a rebondi. Sur la pierre chaude. Victorina pose le ballon dans le panier. Le panier sent le bois.</t>
+          <t>Maman sort le ballon du bac. Il est un peu poudreux. Le ballon, maintenant ! Nino court trop, tout de suite. Il saute vers le ballon. À moi ! Le ballon roule sous le drap. Il est dessous ! Victorina avance les mains, trop vite. Puis elle s'arrête net. Victorina refuse de foncer, cette fois. Ses mains se ferment, puis s'ouvrent. Personne ne dit la suite. Elle observe le ballon, un instant. Elle écoute le clap clap du linge. Sur le bois, un éclat de piquet luit. Là, sur le piquet. Tu tends les mains, Nino ? Nino ne dit rien. Il souffle, puis tend les mains. Oui. On soulève le drap ? Oui, papa. Le drap sent le savon. Le ballon est là, un peu tiède. Victorina le pose près de Nino. Nino le rend, sans courir. Poumf. Poumf. Le ballon est bien gonflé ? Oui, papa. La pierre est chaude, Nino ? Un peu. Ils se passent le ballon, tout près. L'herbe chatouille les genoux. C'est plus facile. Le drap est sec ? Oui, papa. Un rayon passe entre les draps. Il allume le piquet.</t>
         </is>
       </c>
       <c r="F5" s="2" t="inlineStr">
         <is>
-          <t>On rentre ? Oui, maman. Victorina porte le ballon. Nino ramasse la pince rouge. Vous vous dites merci ? Merci, Nino. Merci. Le linge fait encore clap clap. Le ballon a rebondi. Sur la pierre chaude. Victorina pose le ballon dans le panier. Le panier sent le bois.</t>
+          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;Maman sort le ballon du bac. Il est un peu poudreux. Le ballon, maintenant ! Nino court trop, tout de suite. Il saute vers le ballon. À moi ! Le ballon roule sous le drap. Il est dessous ! Victorina avance les mains, trop vite. Puis elle s'arrête net. Victorina refuse de foncer, cette fois. Ses mains se ferment, puis s'ouvrent. Personne ne dit la suite. Elle observe le ballon, un instant. Elle écoute le clap clap du linge. Sur le bois, un &lt;emphasis level="moderate"&gt;éclat de piquet&lt;/emphasis&gt; luit. Là, sur le piquet. Tu tends les mains, Nino ? Nino ne dit rien. Il souffle, puis tend les mains. Oui. On soulève le drap ? Oui, papa. Le drap sent le savon. Le ballon est là, un peu tiède. Victorina le pose près de Nino. Nino le rend, sans courir. Poumf. Poumf. Le ballon est bien gonflé ? Oui, papa. La pierre est chaude, Nino ? Un peu. Ils se passent le ballon, tout près. L'herbe chatouille les genoux. C'est plus facile. Le drap est sec ? Oui, papa. Un rayon passe entre les draps. Il allume le piquet.&lt;/prosody&gt;&lt;break time="480ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G5" s="2" t="inlineStr">
         <is>
-          <t>&lt;slow&gt;Maman dit : on rentre. Sara porte le cerceau. Adam porte le ballon. Ils se disent merci.&lt;/slow&gt; [pause]</t>
+          <t>Maman sort le ballon du bac. Il est un peu poudreux. Le ballon, maintenant ! Nino court trop, tout de suite. Il saute vers le ballon. À moi ! Le ballon roule sous le drap. Il est dessous ! Victorina avance les mains, trop vite. Puis elle s'arrête net. Victorina refuse de foncer, cette fois. Ses mains se ferment, puis s'ouvrent. Personne ne dit la suite. Elle observe le ballon, un instant. Elle écoute le clap clap du linge. Sur le bois, un &lt;emphasis&gt;éclat de piquet&lt;/emphasis&gt; luit. Là, sur le piquet. Tu tends les mains, Nino ? Nino ne dit rien. Il souffle, puis tend les mains. Oui. On soulève le drap ? Oui, papa. Le drap sent le savon. Le ballon est là, un peu tiède. Victorina le pose près de Nino. Nino le rend, sans courir. Poumf. Poumf. Le ballon est bien gonflé ? Oui, papa. La pierre est chaude, Nino ? Un peu. Ils se passent le ballon, tout près. L'herbe chatouille les genoux. C'est plus facile. Le drap est sec ? Oui, papa. Un rayon passe entre les draps. Il allume le piquet. [pause]</t>
         </is>
       </c>
       <c r="H5" s="2" t="inlineStr"/>
@@ -1851,18 +1883,18 @@
         </is>
       </c>
       <c r="Y5" s="2" t="n">
-        <v>118</v>
+        <v>128</v>
       </c>
       <c r="Z5" s="2" t="inlineStr">
         <is>
-          <t>slow</t>
+          <t>medium</t>
         </is>
       </c>
       <c r="AA5" s="2" t="n">
-        <v>0.86</v>
+        <v>0.92</v>
       </c>
       <c r="AB5" s="2" t="n">
-        <v>1.28</v>
+        <v>1.18</v>
       </c>
       <c r="AC5" s="2" t="inlineStr">
         <is>
@@ -1883,28 +1915,32 @@
       <c r="AG5" s="2" t="n">
         <v>0</v>
       </c>
-      <c r="AH5" s="2" t="inlineStr"/>
+      <c r="AH5" s="2" t="inlineStr">
+        <is>
+          <t>éclat de piquet</t>
+        </is>
+      </c>
       <c r="AI5" s="2" t="n">
         <v>200</v>
       </c>
       <c r="AJ5" s="2" t="n">
-        <v>450</v>
+        <v>480</v>
       </c>
       <c r="AK5" s="2" t="n">
-        <v>380</v>
+        <v>280</v>
       </c>
       <c r="AL5" s="2" t="inlineStr">
         <is>
-          <t>calm</t>
+          <t>lively</t>
         </is>
       </c>
       <c r="AM5" s="2" t="inlineStr">
         <is>
-          <t>level</t>
+          <t>dynamic</t>
         </is>
       </c>
       <c r="AN5" s="2" t="n">
-        <v>0.333</v>
+        <v>0.35</v>
       </c>
       <c r="AO5" s="2" t="inlineStr"/>
       <c r="AP5" s="2" t="inlineStr">
@@ -1913,10 +1949,10 @@
         </is>
       </c>
       <c r="AQ5" s="2" t="n">
-        <v>0.86</v>
+        <v>0.92</v>
       </c>
       <c r="AR5" s="2" t="n">
-        <v>0.86</v>
+        <v>0.92</v>
       </c>
       <c r="AS5" s="2" t="n">
         <v>100</v>
@@ -1925,23 +1961,60 @@
         <v>50</v>
       </c>
       <c r="AU5" s="2" t="n">
-        <v>12</v>
-      </c>
-      <c r="AV5" s="2" t="inlineStr"/>
+        <v>8</v>
+      </c>
+      <c r="AV5" s="2" t="inlineStr">
+        <is>
+          <t>arc=action; intention=entraîner; emotion=élan puis prudence; intensite=2; destinataire=enfant; sous_texte=le_ballon_sous_le_drap_elle_s_arrete; tempo=un peu vif puis posé; sourire=léger; respiration=courte</t>
+        </is>
+      </c>
       <c r="AW5" t="inlineStr">
         <is>
-          <t>maman|On rentre ?
-enfant-f|Oui, maman.
-narrateur|Victorina porte le ballon.
-narrateur|Nino ramasse la pince rouge.
-papa|Vous vous dites merci ?
-enfant-f|Merci, Nino.
-enfant-m|Merci.
-narrateur|Le linge fait encore clap clap.
-maman|Le ballon a rebondi.
-papa|Sur la pierre chaude.
-narrateur|Victorina pose le ballon dans le panier.
-narrateur|Le panier sent le bois.</t>
+          <t>narrateur|Maman sort le ballon du bac.
+narrateur|Il est un peu poudreux.
+enfant-f|Le ballon, maintenant !
+narrateur|Nino court trop, tout de suite.
+narrateur|Il saute vers le ballon.
+copain|À moi !
+narrateur|Le ballon roule sous le drap.
+enfant-f|Il est dessous !
+narrateur|Victorina avance les mains, trop vite.
+narrateur|Puis elle s'arrête net.
+narrateur|Victorina refuse de foncer, cette fois.
+narrateur|Ses mains se ferment, puis s'ouvrent.
+narrateur|Personne ne dit la suite.
+narrateur|Elle observe le ballon, un instant.
+narrateur|Elle écoute le clap clap du linge.
+narrateur|Sur le bois, un éclat de piquet luit.
+enfant-f|Là, sur le piquet.
+enfant-f|Tu tends les mains, Nino ?
+narrateur|Nino ne dit rien.
+narrateur|Il souffle, puis tend les mains.
+copain|Oui.
+papa|On soulève le drap ?
+enfant-f|Oui, papa.
+narrateur|Le drap sent le savon.
+narrateur|Le ballon est là, un peu tiède.
+narrateur|Victorina le pose près de Nino.
+narrateur|Nino le rend, sans courir.
+enfant-f|Poumf.
+copain|Poumf.
+papa|Le ballon est bien gonflé ?
+enfant-f|Oui, papa.
+maman|La pierre est chaude, Nino ?
+copain|Un peu.
+narrateur|Ils se passent le ballon, tout près.
+narrateur|L'herbe chatouille les genoux.
+enfant-f|C'est plus facile.
+papa|Le drap est sec ?
+enfant-f|Oui, papa.
+maman|Un rayon passe entre les draps.
+enfant-f|Il allume le piquet.</t>
+        </is>
+      </c>
+      <c r="AX5" t="inlineStr">
+        <is>
+          <t>enfants_parc</t>
         </is>
       </c>
     </row>
@@ -1968,17 +2041,17 @@
       </c>
       <c r="E6" s="2" t="inlineStr">
         <is>
-          <t>La pierre est encore chaude. Le ballon dort dans le panier. Il rebondira demain. Sur la pierre.</t>
+          <t>Ils restent près du piquet. Maman essuie un peu d'herbe. Le cerceau a tourné, papa. Tu l'as vu, toi ? Oui, près du linge. On est bien, ici. Victorina tapote le ballon du doigt. Il a une trace de savon. Tu la vois, la trace ? Oui, maman. Le ballon est resté, Victorina. Oui, avec Nino. Le ballon est resté. Ça sent le savon, un peu tiède. Et le linge, maman. Oui, dans l'air. Le cerceau reste dans l'herbe. Un éclat de piquet tient sur le bois.</t>
         </is>
       </c>
       <c r="F6" s="2" t="inlineStr">
         <is>
-          <t>La pierre est encore chaude. Le ballon dort dans le panier. Il rebondira demain. Sur la pierre.</t>
+          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="-2st"&gt;Ils restent près du piquet. Maman essuie un peu d'herbe. Le cerceau a tourné, papa. Tu l'as vu, toi ? Oui, près du linge. On est bien, ici. Victorina tapote le ballon du doigt. Il a une trace de savon. Tu la vois, la trace ? Oui, maman. Le ballon est resté, Victorina. Oui, avec Nino. Le ballon est resté. Ça sent le savon, un peu tiède. Et le linge, maman. Oui, dans l'air. Le cerceau reste dans l'herbe. Un &lt;emphasis level="moderate"&gt;éclat de piquet&lt;/emphasis&gt; tient sur le bois.&lt;/prosody&gt;&lt;break time="980ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G6" s="2" t="inlineStr">
         <is>
-          <t>&lt;lower-pitch&gt;&lt;soft&gt;&lt;slow&gt;L'histoire est finie.&lt;/slow&gt;&lt;/soft&gt;&lt;/lower-pitch&gt; [pause]</t>
+          <t>&lt;low-pitch&gt;&lt;soft&gt;&lt;slow&gt;Ils restent près du piquet. Maman essuie un peu d'herbe. Le cerceau a tourné, papa. Tu l'as vu, toi ? Oui, près du linge. On est bien, ici. Victorina tapote le ballon du doigt. Il a une trace de savon. Tu la vois, la trace ? Oui, maman. Le ballon est resté, Victorina. Oui, avec Nino. Le ballon est resté. Ça sent le savon, un peu tiède. Et le linge, maman. Oui, dans l'air. Le cerceau reste dans l'herbe. Un &lt;emphasis&gt;éclat de piquet&lt;/emphasis&gt; tient sur le bois.&lt;/slow&gt;&lt;/soft&gt;&lt;/low-pitch&gt; [long-pause]</t>
         </is>
       </c>
       <c r="H6" s="2" t="inlineStr"/>
@@ -2025,7 +2098,7 @@
         </is>
       </c>
       <c r="Y6" s="2" t="n">
-        <v>106</v>
+        <v>102</v>
       </c>
       <c r="Z6" s="2" t="inlineStr">
         <is>
@@ -2033,10 +2106,10 @@
         </is>
       </c>
       <c r="AA6" s="2" t="n">
-        <v>0.82</v>
+        <v>0.8</v>
       </c>
       <c r="AB6" s="2" t="n">
-        <v>1.4</v>
+        <v>1.36</v>
       </c>
       <c r="AC6" s="2" t="inlineStr">
         <is>
@@ -2045,12 +2118,12 @@
       </c>
       <c r="AD6" s="2" t="inlineStr">
         <is>
-          <t>low</t>
+          <t>-2st</t>
         </is>
       </c>
       <c r="AE6" s="2" t="inlineStr">
         <is>
-          <t>lower-pitch</t>
+          <t>low-pitch</t>
         </is>
       </c>
       <c r="AF6" s="2" t="inlineStr">
@@ -2059,14 +2132,18 @@
         </is>
       </c>
       <c r="AG6" s="2" t="n">
-        <v>-2</v>
-      </c>
-      <c r="AH6" s="2" t="inlineStr"/>
+        <v>-3</v>
+      </c>
+      <c r="AH6" s="2" t="inlineStr">
+        <is>
+          <t>éclat de piquet</t>
+        </is>
+      </c>
       <c r="AI6" s="2" t="n">
         <v>200</v>
       </c>
       <c r="AJ6" s="2" t="n">
-        <v>600</v>
+        <v>980</v>
       </c>
       <c r="AK6" s="2" t="n">
         <v>380</v>
@@ -2078,11 +2155,11 @@
       </c>
       <c r="AM6" s="2" t="inlineStr">
         <is>
-          <t>fall</t>
+          <t>falling</t>
         </is>
       </c>
       <c r="AN6" s="2" t="n">
-        <v>0.333</v>
+        <v>0.29</v>
       </c>
       <c r="AO6" s="2" t="inlineStr"/>
       <c r="AP6" s="2" t="inlineStr">
@@ -2091,27 +2168,45 @@
         </is>
       </c>
       <c r="AQ6" s="2" t="n">
-        <v>0.82</v>
+        <v>0.8</v>
       </c>
       <c r="AR6" s="2" t="n">
-        <v>0.82</v>
+        <v>0.8</v>
       </c>
       <c r="AS6" s="2" t="n">
-        <v>80</v>
+        <v>82</v>
       </c>
       <c r="AT6" s="2" t="n">
-        <v>35</v>
+        <v>42</v>
       </c>
       <c r="AU6" s="2" t="n">
         <v>12</v>
       </c>
-      <c r="AV6" s="2" t="inlineStr"/>
+      <c r="AV6" s="2" t="inlineStr">
+        <is>
+          <t>arc=retour; intention=refermer; emotion=tendresse_et_fierté_calme; intensite=1; destinataire=enfant; sous_texte=l_eclat_du_debut_tient_sur_le_bois; tempo=très posé; sourire=léger; respiration=ample</t>
+        </is>
+      </c>
       <c r="AW6" t="inlineStr">
         <is>
-          <t>narrateur|La pierre est encore chaude.
-narrateur|Le ballon dort dans le panier.
-papa|Il rebondira demain.
-enfant-f|Sur la pierre.</t>
+          <t>narrateur|Ils restent près du piquet.
+narrateur|Maman essuie un peu d'herbe.
+enfant-f|Le cerceau a tourné, papa.
+papa|Tu l'as vu, toi ?
+enfant-f|Oui, près du linge.
+maman|On est bien, ici.
+narrateur|Victorina tapote le ballon du doigt.
+enfant-f|Il a une trace de savon.
+maman|Tu la vois, la trace ?
+enfant-f|Oui, maman.
+papa|Le ballon est resté, Victorina.
+enfant-f|Oui, avec Nino.
+copain|Le ballon est resté.
+narrateur|Ça sent le savon, un peu tiède.
+enfant-f|Et le linge, maman.
+maman|Oui, dans l'air.
+narrateur|Le cerceau reste dans l'herbe.
+narrateur|Un éclat de piquet tient sur le bois.</t>
         </is>
       </c>
     </row>
@@ -2132,7 +2227,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A12"/>
+  <dimension ref="A1:A13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="100" customWidth="1" min="1" max="1"/>
@@ -2217,6 +2312,13 @@
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
+        <is>
+          <t>F-NAR-008 récit, pas une leçon en puces</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
         <is>
           <t>F-NAR-008 récit, pas une leçon en puces</t>
         </is>

</xml_diff>